<commit_message>
auto(MT): 3h refresh 2026-05-18T16:07Z
</commit_message>
<xml_diff>
--- a/daily_report_mt_2026-05-18.xlsx
+++ b/daily_report_mt_2026-05-18.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,8 +32,12 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +59,11 @@
         <fgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -68,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -79,6 +88,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,22 +456,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="9" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="7" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -530,13 +542,246 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No ads detected as removed today.</t>
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>John Baptist Camilleri</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>John Baptist Camilleri</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>971816796212886</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>993445096523240</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="n"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>10,000–14,999</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18 15:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>George Vital Zammit</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">George Vital Zammit Kandidat PN </t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1162563556930834</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>864621386654273</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-05-14</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>20,000–24,999</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-05-18 15:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Alex Borg</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>PN</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr"/>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Leone Sciberras</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>346098823146420</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>1368678455314097</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="n"/>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>2,000–2,999</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>2026-05-18 15:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Olaf McKay</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Olaf McKay</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>328880766964335</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>1732358601287330</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>3,000–3,999</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0–99</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>2026-05-18 15:59</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>